<commit_message>
[Lab1]: fix Script, add comments in Excel
</commit_message>
<xml_diff>
--- a/Lab1/Solver.xlsx
+++ b/Lab1/Solver.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Personal papka\МетОпт\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\optimization-methods\Lab1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A5EA33-07B9-4694-B7E4-D9C3AC76BC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA9EF5E-362E-44B5-A726-70B625B518C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,33 +17,33 @@
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">Лист1!$B$6:$E$6</definedName>
-    <definedName name="solver_cvg" localSheetId="0" hidden="1">"""""""0,0001"""""""</definedName>
+    <definedName name="solver_cvg" localSheetId="0" hidden="1">"""""""""""""""0,0001"""""""""""""""</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Лист1!$B$6:$E$6</definedName>
-    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Лист1!$G$3</definedName>
-    <definedName name="solver_lhs3" localSheetId="0" hidden="1">Лист1!$G$4</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Лист1!$G$3</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">Лист1!$G$4</definedName>
+    <definedName name="solver_lhs3" localSheetId="0" hidden="1">Лист1!$G$5</definedName>
     <definedName name="solver_lhs4" localSheetId="0" hidden="1">Лист1!$G$5</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="0" hidden="1">"""""""0,075"""""""</definedName>
+    <definedName name="solver_mrt" localSheetId="0" hidden="1">"""""""""""""""0,075"""""""""""""""</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
-    <definedName name="solver_num" localSheetId="0" hidden="1">4</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Лист1!$G$2</definedName>
-    <definedName name="solver_pre" localSheetId="0" hidden="1">"""""""0,000001"""""""</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">"""""""""""""""0,000001"""""""""""""""</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_rel1" localSheetId="0" hidden="1">4</definedName>
-    <definedName name="solver_rel2" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_rel3" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rel3" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_rel4" localSheetId="0" hidden="1">3</definedName>
-    <definedName name="solver_rhs1" localSheetId="0" hidden="1">"целое"</definedName>
-    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Лист1!$I$3</definedName>
-    <definedName name="solver_rhs3" localSheetId="0" hidden="1">Лист1!$I$4</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Лист1!$I$3</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">Лист1!$I$4</definedName>
+    <definedName name="solver_rhs3" localSheetId="0" hidden="1">Лист1!$I$5</definedName>
     <definedName name="solver_rhs4" localSheetId="0" hidden="1">Лист1!$I$5</definedName>
     <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
@@ -181,11 +181,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -202,6 +202,1395 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>62120</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>33474</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>6408</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>25149</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82BA8B45-554D-4C71-9022-F2EDB0FB6E14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1380435" y="5831300"/>
+          <a:ext cx="4568745" cy="4436675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="43000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>6902</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>22087</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>362052</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>186017</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Рисунок 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B86D581-CEE6-4B9A-A524-E27A48431E85}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="400326" y="1954696"/>
+          <a:ext cx="3592269" cy="1130234"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="43000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>114852</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>85587</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>260902</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>170898</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="TextBox 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC99FB5F-3B79-4F25-B90E-2AB8A429BA10}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="508276" y="1631674"/>
+          <a:ext cx="3383169" cy="278572"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>Сюда</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t> вводим коэффициенты матрицы ограничений</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>6902</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>151848</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>362052</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>177544</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Рисунок 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81A6BBD3-5D4C-45F6-8465-9E687235D027}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4562337" y="1891196"/>
+          <a:ext cx="3592269" cy="1185261"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="43000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>146602</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>22087</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>292652</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>104637</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="TextBox 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58FDD678-057A-4133-A77E-74B624E88002}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4702037" y="1568174"/>
+          <a:ext cx="3383169" cy="275811"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>Сюда</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t> вводим коэффициенты целевой функции</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>20705</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>165652</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>383586</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>137841</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Рисунок 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9E74F33-38EE-4311-A53C-F810B9BCC233}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="414129" y="3837609"/>
+          <a:ext cx="3600000" cy="1131754"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="43000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>158750</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>27610</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>112921</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="TextBox 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38FB9050-0FA6-468A-BE1C-739409AF6147}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="552174" y="3506306"/>
+          <a:ext cx="3383169" cy="278572"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>Здесь</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t> будут подобранные </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>x1, x2, x3, x4</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>165652</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>48315</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>66087</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>35753</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Рисунок 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11605F21-D0EC-4000-BF06-28941A45B92A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4721087" y="4300054"/>
+          <a:ext cx="3600000" cy="1147003"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="43000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>290444</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>6902</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>436494</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>179457</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="TextBox 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B440660-7BA5-41A7-8980-795F0191437B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4845879" y="3292337"/>
+          <a:ext cx="3383169" cy="945598"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>В</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t> этих ячейках записана формула, которая считает значение функции (целевой или ограничивающей) при конкретных </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>x1, x2, x3, x4</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>. Если точнее - считается скалярное произведение вектора функции на вектор переменных </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>x</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>55217</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>69022</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>448642</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="TextBox 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA38494B-7155-4DBE-849E-214F39FFE92C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3223315" y="2967935"/>
+          <a:ext cx="855870" cy="282989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Рисунок 1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>138043</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>69022</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>69022</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="TextBox 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E3B84E0-4793-4AFD-A89B-3449FB23177E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7468152" y="2967935"/>
+          <a:ext cx="855870" cy="282989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Рисунок 2</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>186358</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>69022</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>117337</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="TextBox 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{881F3206-F197-44F1-A7E4-704BFCFAAE66}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3354456" y="4900544"/>
+          <a:ext cx="855870" cy="282989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Рисунок 3</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>289891</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>117338</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>220870</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>13805</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="TextBox 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3480BC82-6406-484A-95BF-CD231F6C5A98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7620000" y="5335381"/>
+          <a:ext cx="855870" cy="282989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Рисунок 4</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>262835</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>138597</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>193813</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>35064</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="TextBox 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4D10E80-2AAD-474B-9A10-2493515633CF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5280715" y="10188162"/>
+          <a:ext cx="855870" cy="282989"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Рисунок 5</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>140805</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>132521</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>252557</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>151534</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="TextBox 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9556D2D6-D474-44CD-A524-254558CD897E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6079498" y="6886612"/>
+          <a:ext cx="3344479" cy="1332308"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100"/>
+            <a:t>Изменяем значения </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>x1,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> x2, x3, x4 </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>так, чтобы ячейка </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>G2 (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>где считается знаечение ЦФ при конкретных </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>x1, x2, x3, x4) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>содержала максимальное значение, </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>учитывая ограничения значений функций-ограничений (значения считаются в </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>G3-5</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>)</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>. </a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>Ставим галочку, что все </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>x </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>положительные. </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1100" baseline="0"/>
+            <a:t>Выбираем метод решения симплекс-методом.</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>339147</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>43295</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>194830</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>79375</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="28" name="Прямая со стрелкой 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66234AFB-F3FC-4832-B079-7E70921FB38F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="2121477" y="6797386"/>
+          <a:ext cx="4012046" cy="223694"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>57728</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>144319</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>209262</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>50513</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="29" name="Прямая со стрелкой 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47F97405-24B9-4C67-B4B1-AB15D0DCB75E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="3687330" y="6147955"/>
+          <a:ext cx="2460625" cy="1031876"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>447386</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>28863</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>194831</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>57729</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="31" name="Прямая со стрелкой 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B22C76C-394A-4369-BAAF-05B0D3F8E22F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="2229716" y="7345795"/>
+          <a:ext cx="3903808" cy="216479"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7215</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>180398</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>202046</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>115455</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="33" name="Прямая со стрелкой 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{159466CE-2765-4E6C-A176-392F1228870C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="1789545" y="7872557"/>
+          <a:ext cx="4351194" cy="497898"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>346365</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>180398</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>50512</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="36" name="Прямая со стрелкой 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67A49181-0356-4A74-805B-C4973874379B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="4437785" y="8067386"/>
+          <a:ext cx="1681306" cy="613353"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -514,9 +1903,9 @@
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="5">
         <f>SUMPRODUCT($B$6:$E$6,B2:E2)</f>
-        <v>19</v>
+        <v>210</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>9</v>
@@ -528,7 +1917,7 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2">
@@ -548,7 +1937,7 @@
       </c>
       <c r="G3" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B3:E3)</f>
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>5</v>
@@ -560,7 +1949,7 @@
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5"/>
+      <c r="A4" s="6"/>
       <c r="B4" s="2">
         <v>0</v>
       </c>
@@ -578,7 +1967,7 @@
       </c>
       <c r="G4" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B4:E4)</f>
-        <v>6</v>
+        <v>120</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>11</v>
@@ -590,7 +1979,7 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="2">
         <v>1</v>
       </c>
@@ -608,7 +1997,7 @@
       </c>
       <c r="G5" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B5:E5)</f>
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>6</v>
@@ -623,17 +2012,17 @@
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6">
-        <v>7</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0</v>
-      </c>
-      <c r="D6" s="6">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6">
-        <v>0</v>
+      <c r="B6" s="5">
+        <v>10</v>
+      </c>
+      <c r="C6" s="5">
+        <v>20</v>
+      </c>
+      <c r="D6" s="5">
+        <v>30</v>
+      </c>
+      <c r="E6" s="5">
+        <v>40</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -775,5 +2164,6 @@
     <mergeCell ref="A3:A5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Lab1]: add solve in Solver.xlsx
</commit_message>
<xml_diff>
--- a/Lab1/Solver.xlsx
+++ b/Lab1/Solver.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\optimization-methods\Lab1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA9EF5E-362E-44B5-A726-70B625B518C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2686D028-8C39-4A76-94C5-E8922729A540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">Лист1!$B$6:$E$6</definedName>
-    <definedName name="solver_cvg" localSheetId="0" hidden="1">"""""""""""""""0,0001"""""""""""""""</definedName>
+    <definedName name="solver_cvg" localSheetId="0" hidden="1">"""""""""""""""""""""""""""""""0,0001"""""""""""""""""""""""""""""""</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
@@ -28,14 +28,14 @@
     <definedName name="solver_lhs4" localSheetId="0" hidden="1">Лист1!$G$5</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
-    <definedName name="solver_mrt" localSheetId="0" hidden="1">"""""""""""""""0,075"""""""""""""""</definedName>
+    <definedName name="solver_mrt" localSheetId="0" hidden="1">"""""""""""""""""""""""""""""""0,075"""""""""""""""""""""""""""""""</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">Лист1!$G$2</definedName>
-    <definedName name="solver_pre" localSheetId="0" hidden="1">"""""""""""""""0,000001"""""""""""""""</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">"""""""""""""""""""""""""""""""0,000001"""""""""""""""""""""""""""""""</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G2" s="5">
         <f>SUMPRODUCT($B$6:$E$6,B2:E2)</f>
-        <v>210</v>
+        <v>19</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>9</v>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="G3" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B3:E3)</f>
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>5</v>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="G4" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B4:E4)</f>
-        <v>120</v>
+        <v>6</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>11</v>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="G5" s="1">
         <f>SUMPRODUCT($B$6:$E$6,B5:E5)</f>
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>6</v>
@@ -2013,16 +2013,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6" s="5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D6" s="5">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E6" s="5">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>

</xml_diff>